<commit_message>
Update BFPIE and Carbon Tax Rate
</commit_message>
<xml_diff>
--- a/InputData/land/BLAPE/cn-BAU LULUCF Anthropogenic Pollutant Emissions.xlsx
+++ b/InputData/land/BLAPE/cn-BAU LULUCF Anthropogenic Pollutant Emissions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\EPS\Github Push\China\eps-china2019-smart-trans\InputData\land\BLAPE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F296BE90-28CB-412F-B1CB-F4B0343B626B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AE78FFB-70F2-470A-B544-BD5B71C8E92D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="165" yWindow="2400" windowWidth="21600" windowHeight="11385" tabRatio="833" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="833" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="4" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1364" uniqueCount="827">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1367" uniqueCount="827">
   <si>
     <t>单位：万亩</t>
   </si>
@@ -3865,21 +3865,6 @@
   </si>
   <si>
     <r>
-      <t>75</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="宋体"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>、2</t>
-    </r>
-    <phoneticPr fontId="27" type="noConversion"/>
-  </si>
-  <si>
-    <r>
       <rPr>
         <sz val="10"/>
         <rFont val="Times New Roman"/>
@@ -4074,6 +4059,10 @@
       </rPr>
       <t>其他生物质</t>
     </r>
+  </si>
+  <si>
+    <t>NE</t>
+    <phoneticPr fontId="27" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -4086,7 +4075,7 @@
     <numFmt numFmtId="178" formatCode="0_ "/>
     <numFmt numFmtId="179" formatCode="0.0_ "/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="33">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4308,12 +4297,6 @@
     <font>
       <sz val="10"/>
       <name val="SimSun"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="宋体"/>
-      <family val="2"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -5570,11 +5553,11 @@
         <v>336</v>
       </c>
       <c r="B2">
-        <f>温室气体排放清单!K9*10^10</f>
+        <f>温室气体排放清单!N9*10^10</f>
         <v>-1342629000000000</v>
       </c>
       <c r="C2">
-        <f>温室气体排放清单!N9*10^10</f>
+        <f>温室气体排放清单!Q9*10^10</f>
         <v>-1346499000000000</v>
       </c>
       <c r="D2">
@@ -6763,11 +6746,11 @@
         <v>345</v>
       </c>
       <c r="B11">
-        <f>温室气体排放清单!L9*10^10</f>
+        <f>温室气体排放清单!O9*10^10</f>
         <v>1398000000000</v>
       </c>
       <c r="C11">
-        <f>温室气体排放清单!O9*10^10</f>
+        <f>温室气体排放清单!R9*10^10</f>
         <v>1110000000000</v>
       </c>
       <c r="D11">
@@ -11912,42 +11895,47 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2DE32B2-125A-4EC5-B7EE-D8C69A079B2B}">
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:S17"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="16" width="10" customWidth="1"/>
+    <col min="2" max="19" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:19">
       <c r="A1" s="17"/>
       <c r="B1" s="129">
-        <v>2017</v>
+        <v>2005</v>
       </c>
       <c r="C1" s="129"/>
       <c r="D1" s="129"/>
       <c r="E1" s="129">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="F1" s="129"/>
       <c r="G1" s="129"/>
-      <c r="H1" s="129" t="s">
-        <v>804</v>
+      <c r="H1" s="129">
+        <v>2018</v>
       </c>
       <c r="I1" s="129"/>
       <c r="J1" s="129"/>
       <c r="K1" s="129" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="L1" s="129"/>
       <c r="M1" s="129"/>
-      <c r="N1" s="129">
-        <v>2021</v>
+      <c r="N1" s="129" t="s">
+        <v>805</v>
       </c>
       <c r="O1" s="129"/>
       <c r="P1" s="129"/>
-    </row>
-    <row r="2" spans="1:16" ht="14.25">
+      <c r="Q1" s="129">
+        <v>2021</v>
+      </c>
+      <c r="R1" s="129"/>
+      <c r="S1" s="129"/>
+    </row>
+    <row r="2" spans="1:19" ht="14.25">
       <c r="A2" s="17"/>
       <c r="B2" s="115" t="s">
         <v>806</v>
@@ -11994,567 +11982,674 @@
       <c r="P2" s="115" t="s">
         <v>808</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" ht="14.25">
+      <c r="Q2" s="115" t="s">
+        <v>806</v>
+      </c>
+      <c r="R2" s="115" t="s">
+        <v>807</v>
+      </c>
+      <c r="S2" s="115" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="14.25">
       <c r="A3" s="116" t="s">
         <v>809</v>
       </c>
       <c r="B3" s="117"/>
       <c r="C3" s="117">
-        <v>2470.8000000000002</v>
+        <v>2136.5</v>
       </c>
       <c r="D3" s="117">
-        <v>98.2</v>
+        <v>98.3</v>
       </c>
       <c r="E3" s="117"/>
       <c r="F3" s="117">
-        <v>2136.5</v>
+        <v>2470.8000000000002</v>
       </c>
       <c r="G3" s="117">
-        <v>98.3</v>
+        <v>98.2</v>
       </c>
       <c r="H3" s="117"/>
       <c r="I3" s="117">
-        <v>2384.6</v>
+        <v>2136.5</v>
       </c>
       <c r="J3" s="117">
-        <v>94.3</v>
+        <v>98.3</v>
       </c>
       <c r="K3" s="117"/>
       <c r="L3" s="117">
-        <v>2372</v>
+        <v>2384.6</v>
       </c>
       <c r="M3" s="117">
-        <v>94.6</v>
+        <v>94.3</v>
       </c>
       <c r="N3" s="117"/>
       <c r="O3" s="117">
+        <v>2372</v>
+      </c>
+      <c r="P3" s="117">
+        <v>94.6</v>
+      </c>
+      <c r="Q3" s="117"/>
+      <c r="R3" s="117">
         <v>2427.9</v>
       </c>
-      <c r="P3" s="117">
+      <c r="S3" s="117">
         <v>94.9</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="14.25">
+    <row r="4" spans="1:19" ht="14.25">
       <c r="A4" s="116" t="s">
         <v>810</v>
       </c>
       <c r="B4" s="117"/>
       <c r="C4" s="117">
-        <v>1112.3</v>
+        <v>1120.4000000000001</v>
       </c>
       <c r="D4" s="117"/>
       <c r="E4" s="117"/>
       <c r="F4" s="117">
-        <v>1120.4000000000001</v>
+        <v>1112.3</v>
       </c>
       <c r="G4" s="117"/>
       <c r="H4" s="117"/>
       <c r="I4" s="117">
-        <v>1084.0999999999999</v>
+        <v>1120.4000000000001</v>
       </c>
       <c r="J4" s="117"/>
       <c r="K4" s="117"/>
       <c r="L4" s="117">
-        <v>1124.2</v>
+        <v>1084.0999999999999</v>
       </c>
       <c r="M4" s="117"/>
       <c r="N4" s="117"/>
       <c r="O4" s="117">
+        <v>1124.2</v>
+      </c>
+      <c r="P4" s="117"/>
+      <c r="Q4" s="117"/>
+      <c r="R4" s="117">
         <v>1151.8</v>
       </c>
-      <c r="P4" s="117"/>
-    </row>
-    <row r="5" spans="1:16" ht="14.25">
+      <c r="S4" s="117"/>
+    </row>
+    <row r="5" spans="1:19" ht="14.25">
       <c r="A5" s="116" t="s">
         <v>811</v>
       </c>
       <c r="B5" s="117"/>
       <c r="C5" s="117">
-        <v>354.8</v>
+        <v>240.4</v>
       </c>
       <c r="D5" s="117">
-        <v>22</v>
+        <v>27.2</v>
       </c>
       <c r="E5" s="117"/>
       <c r="F5" s="117">
-        <v>240.4</v>
+        <v>354.8</v>
       </c>
       <c r="G5" s="117">
-        <v>27.2</v>
+        <v>22</v>
       </c>
       <c r="H5" s="117"/>
       <c r="I5" s="117">
-        <v>346.1</v>
+        <v>240.4</v>
       </c>
       <c r="J5" s="117">
-        <v>21.7</v>
+        <v>27.2</v>
       </c>
       <c r="K5" s="117"/>
       <c r="L5" s="117">
-        <v>344.7</v>
+        <v>346.1</v>
       </c>
       <c r="M5" s="117">
-        <v>22.2</v>
+        <v>21.7</v>
       </c>
       <c r="N5" s="117"/>
       <c r="O5" s="117">
+        <v>344.7</v>
+      </c>
+      <c r="P5" s="117">
+        <v>22.2</v>
+      </c>
+      <c r="Q5" s="117"/>
+      <c r="R5" s="117">
         <v>375.3</v>
       </c>
-      <c r="P5" s="117">
+      <c r="S5" s="117">
         <v>22.7</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="14.25">
+    <row r="6" spans="1:19" ht="14.25">
       <c r="A6" s="116" t="s">
         <v>812</v>
       </c>
       <c r="B6" s="117"/>
       <c r="C6" s="117">
-        <v>962.8</v>
+        <v>755</v>
       </c>
       <c r="D6" s="117"/>
       <c r="E6" s="117"/>
       <c r="F6" s="117">
-        <v>755</v>
+        <v>962.8</v>
       </c>
       <c r="G6" s="117"/>
       <c r="H6" s="117"/>
       <c r="I6" s="117">
-        <v>932.9</v>
+        <v>755</v>
       </c>
       <c r="J6" s="117"/>
       <c r="K6" s="117"/>
       <c r="L6" s="117">
-        <v>884.9</v>
+        <v>932.9</v>
       </c>
       <c r="M6" s="117"/>
       <c r="N6" s="117"/>
       <c r="O6" s="117">
+        <v>884.9</v>
+      </c>
+      <c r="P6" s="117"/>
+      <c r="Q6" s="117"/>
+      <c r="R6" s="117">
         <v>885.1</v>
       </c>
-      <c r="P6" s="117"/>
-    </row>
-    <row r="7" spans="1:16" ht="14.25">
+      <c r="S6" s="117"/>
+    </row>
+    <row r="7" spans="1:19" ht="14.25">
       <c r="A7" s="116" t="s">
         <v>813</v>
       </c>
       <c r="B7" s="117"/>
       <c r="C7" s="117"/>
-      <c r="D7" s="117" t="s">
-        <v>814</v>
+      <c r="D7" s="117">
+        <v>70.599999999999994</v>
       </c>
       <c r="E7" s="117"/>
       <c r="F7" s="117"/>
       <c r="G7" s="117">
-        <v>70.599999999999994</v>
+        <v>75.2</v>
       </c>
       <c r="H7" s="117"/>
       <c r="I7" s="117"/>
       <c r="J7" s="117">
-        <v>72</v>
+        <v>70.599999999999994</v>
       </c>
       <c r="K7" s="117"/>
       <c r="L7" s="117"/>
       <c r="M7" s="117">
-        <v>71.900000000000006</v>
+        <v>72</v>
       </c>
       <c r="N7" s="117"/>
       <c r="O7" s="117"/>
       <c r="P7" s="117">
+        <v>71.900000000000006</v>
+      </c>
+      <c r="Q7" s="117"/>
+      <c r="R7" s="117"/>
+      <c r="S7" s="117">
         <v>71.8</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="14.25">
+    <row r="8" spans="1:19" ht="14.25">
       <c r="A8" s="116" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="B8" s="117"/>
       <c r="C8" s="117">
-        <v>41</v>
+        <v>20.7</v>
       </c>
       <c r="D8" s="117">
-        <v>1.1000000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="E8" s="117"/>
       <c r="F8" s="117">
-        <v>20.7</v>
+        <v>41</v>
       </c>
       <c r="G8" s="117">
-        <v>0.5</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H8" s="117"/>
       <c r="I8" s="117">
-        <v>21.6</v>
+        <v>20.7</v>
       </c>
       <c r="J8" s="117">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="K8" s="117"/>
       <c r="L8" s="117">
-        <v>18.2</v>
+        <v>21.6</v>
       </c>
       <c r="M8" s="117">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="N8" s="117"/>
       <c r="O8" s="117">
+        <v>18.2</v>
+      </c>
+      <c r="P8" s="117">
+        <v>0.5</v>
+      </c>
+      <c r="Q8" s="117"/>
+      <c r="R8" s="117">
         <v>15.7</v>
       </c>
-      <c r="P8" s="117">
+      <c r="S8" s="117">
         <v>0.4</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="36.75">
+    <row r="9" spans="1:19" ht="36.75">
       <c r="A9" s="118" t="s">
+        <v>815</v>
+      </c>
+      <c r="B9" s="117">
+        <v>-72866.7</v>
+      </c>
+      <c r="C9" s="117">
+        <v>63.2</v>
+      </c>
+      <c r="D9" s="117">
+        <v>0</v>
+      </c>
+      <c r="E9" s="117">
+        <v>-134171.4</v>
+      </c>
+      <c r="F9" s="117"/>
+      <c r="G9" s="117"/>
+      <c r="H9" s="117">
+        <v>-72866.7</v>
+      </c>
+      <c r="I9" s="117">
+        <v>63.2</v>
+      </c>
+      <c r="J9" s="117">
+        <v>0</v>
+      </c>
+      <c r="K9" s="117">
+        <v>-134047.29999999999</v>
+      </c>
+      <c r="L9" s="117">
+        <v>398.1</v>
+      </c>
+      <c r="M9" s="117">
+        <v>0.1</v>
+      </c>
+      <c r="N9" s="117">
+        <v>-134262.9</v>
+      </c>
+      <c r="O9" s="117">
+        <v>139.80000000000001</v>
+      </c>
+      <c r="P9" s="117">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="117">
+        <v>-134649.9</v>
+      </c>
+      <c r="R9" s="117">
+        <v>111</v>
+      </c>
+      <c r="S9" s="117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="14.25">
+      <c r="A10" s="116" t="s">
         <v>816</v>
       </c>
-      <c r="B9" s="117">
-        <v>-134171.4</v>
-      </c>
-      <c r="C9" s="117"/>
-      <c r="D9" s="117"/>
-      <c r="E9" s="117">
-        <v>-72866.7</v>
-      </c>
-      <c r="F9" s="117">
-        <v>63.2</v>
-      </c>
-      <c r="G9" s="117">
-        <v>0</v>
-      </c>
-      <c r="H9" s="117">
-        <v>-134047.29999999999</v>
-      </c>
-      <c r="I9" s="117">
-        <v>398.1</v>
-      </c>
-      <c r="J9" s="117">
+      <c r="B10" s="117">
+        <v>-55120.5</v>
+      </c>
+      <c r="C10" s="117">
+        <v>0.2</v>
+      </c>
+      <c r="D10" s="117">
+        <v>0</v>
+      </c>
+      <c r="E10" s="117">
+        <v>-92842</v>
+      </c>
+      <c r="F10" s="117"/>
+      <c r="G10" s="117"/>
+      <c r="H10" s="117">
+        <v>-55120.5</v>
+      </c>
+      <c r="I10" s="117">
+        <v>0.2</v>
+      </c>
+      <c r="J10" s="117">
+        <v>0</v>
+      </c>
+      <c r="K10" s="117">
+        <v>-96579.199999999997</v>
+      </c>
+      <c r="L10" s="117">
         <v>0.1</v>
       </c>
-      <c r="K9" s="117">
-        <v>-134262.9</v>
-      </c>
-      <c r="L9" s="117">
-        <v>139.80000000000001</v>
-      </c>
-      <c r="M9" s="117">
-        <v>0</v>
-      </c>
-      <c r="N9" s="117">
-        <v>-134649.9</v>
-      </c>
-      <c r="O9" s="117">
-        <v>111</v>
-      </c>
-      <c r="P9" s="117">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="14.25">
-      <c r="A10" s="116" t="s">
+      <c r="M10" s="117">
+        <v>0</v>
+      </c>
+      <c r="N10" s="117">
+        <v>-89559.2</v>
+      </c>
+      <c r="O10" s="117">
+        <v>0</v>
+      </c>
+      <c r="P10" s="117">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="117">
+        <v>-87682.7</v>
+      </c>
+      <c r="R10" s="117">
+        <v>0</v>
+      </c>
+      <c r="S10" s="117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="14.25">
+      <c r="A11" s="116" t="s">
         <v>817</v>
       </c>
-      <c r="B10" s="117">
-        <v>-92842</v>
-      </c>
-      <c r="C10" s="117"/>
-      <c r="D10" s="117"/>
-      <c r="E10" s="117">
-        <v>-55120.5</v>
-      </c>
-      <c r="F10" s="117">
-        <v>0.2</v>
-      </c>
-      <c r="G10" s="117">
-        <v>0</v>
-      </c>
-      <c r="H10" s="117">
-        <v>-96579.199999999997</v>
-      </c>
-      <c r="I10" s="117">
-        <v>0.1</v>
-      </c>
-      <c r="J10" s="117">
-        <v>0</v>
-      </c>
-      <c r="K10" s="117">
-        <v>-89559.2</v>
-      </c>
-      <c r="L10" s="117">
-        <v>0</v>
-      </c>
-      <c r="M10" s="117">
-        <v>0</v>
-      </c>
-      <c r="N10" s="117">
-        <v>-87682.7</v>
-      </c>
-      <c r="O10" s="117">
-        <v>0</v>
-      </c>
-      <c r="P10" s="117">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="14.25">
-      <c r="A11" s="116" t="s">
-        <v>818</v>
-      </c>
       <c r="B11" s="117">
-        <v>-9643.2999999999993</v>
+        <v>-4107.7</v>
       </c>
       <c r="C11" s="117"/>
       <c r="D11" s="117"/>
       <c r="E11" s="117">
-        <v>-4107.7</v>
+        <v>-9643.2999999999993</v>
       </c>
       <c r="F11" s="117"/>
       <c r="G11" s="117"/>
       <c r="H11" s="117">
+        <v>-4107.7</v>
+      </c>
+      <c r="I11" s="117"/>
+      <c r="J11" s="117"/>
+      <c r="K11" s="117">
         <v>-7810</v>
       </c>
-      <c r="I11" s="117" t="s">
-        <v>819</v>
-      </c>
-      <c r="J11" s="117" t="s">
-        <v>819</v>
-      </c>
-      <c r="K11" s="117">
+      <c r="L11" s="117" t="s">
+        <v>818</v>
+      </c>
+      <c r="M11" s="117" t="s">
+        <v>818</v>
+      </c>
+      <c r="N11" s="117">
         <v>-9801.7999999999993</v>
-      </c>
-      <c r="L11" s="117"/>
-      <c r="M11" s="117"/>
-      <c r="N11" s="117">
-        <v>-10616.2</v>
       </c>
       <c r="O11" s="117"/>
       <c r="P11" s="117"/>
-    </row>
-    <row r="12" spans="1:16" ht="14.25">
+      <c r="Q11" s="117">
+        <v>-10616.2</v>
+      </c>
+      <c r="R11" s="117"/>
+      <c r="S11" s="117"/>
+    </row>
+    <row r="12" spans="1:19" ht="14.25">
       <c r="A12" s="116" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B12" s="117">
-        <v>-12101.3</v>
+        <v>-4776.8999999999996</v>
       </c>
       <c r="C12" s="117">
         <v>0.1</v>
       </c>
       <c r="D12" s="117">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="117">
-        <v>-4776.8999999999996</v>
+        <v>-12101.3</v>
       </c>
       <c r="F12" s="117">
         <v>0.1</v>
       </c>
       <c r="G12" s="117">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H12" s="117">
-        <v>-10175.200000000001</v>
+        <v>-4776.8999999999996</v>
       </c>
       <c r="I12" s="117">
         <v>0.1</v>
       </c>
       <c r="J12" s="117">
+        <v>0</v>
+      </c>
+      <c r="K12" s="117">
+        <v>-10175.200000000001</v>
+      </c>
+      <c r="L12" s="117">
         <v>0.1</v>
       </c>
-      <c r="K12" s="117">
+      <c r="M12" s="117">
+        <v>0.1</v>
+      </c>
+      <c r="N12" s="117">
         <v>-7270.7</v>
       </c>
-      <c r="L12" s="117">
-        <v>0</v>
-      </c>
-      <c r="M12" s="117">
-        <v>0</v>
-      </c>
-      <c r="N12" s="117">
+      <c r="O12" s="117">
+        <v>0</v>
+      </c>
+      <c r="P12" s="117">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="117">
         <v>-6408.2</v>
       </c>
-      <c r="O12" s="117">
-        <v>0</v>
-      </c>
-      <c r="P12" s="117">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="14.25">
+      <c r="R12" s="117">
+        <v>0</v>
+      </c>
+      <c r="S12" s="117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="14.25">
       <c r="A13" s="116" t="s">
+        <v>820</v>
+      </c>
+      <c r="B13" s="117">
+        <v>-1373</v>
+      </c>
+      <c r="C13" s="117">
+        <v>62.9</v>
+      </c>
+      <c r="D13" s="117" t="s">
+        <v>826</v>
+      </c>
+      <c r="E13" s="117">
+        <v>-8586.2999999999993</v>
+      </c>
+      <c r="F13" s="117">
+        <v>398.3</v>
+      </c>
+      <c r="G13" s="117"/>
+      <c r="H13" s="117">
+        <v>-1373</v>
+      </c>
+      <c r="I13" s="117">
+        <v>62.9</v>
+      </c>
+      <c r="J13" s="117" t="s">
         <v>821</v>
       </c>
-      <c r="B13" s="117">
-        <v>-8586.2999999999993</v>
-      </c>
-      <c r="C13" s="117">
-        <v>398.3</v>
-      </c>
-      <c r="D13" s="117"/>
-      <c r="E13" s="117">
-        <v>-1373</v>
-      </c>
-      <c r="F13" s="117">
-        <v>62.9</v>
-      </c>
-      <c r="G13" s="117" t="s">
+      <c r="K13" s="117">
+        <v>-8641.7000000000007</v>
+      </c>
+      <c r="L13" s="117">
+        <v>398</v>
+      </c>
+      <c r="M13" s="117" t="s">
+        <v>821</v>
+      </c>
+      <c r="N13" s="117">
+        <v>-2978.8</v>
+      </c>
+      <c r="O13" s="117">
+        <v>139.80000000000001</v>
+      </c>
+      <c r="P13" s="117" t="s">
+        <v>821</v>
+      </c>
+      <c r="Q13" s="117">
+        <v>-2459.9</v>
+      </c>
+      <c r="R13" s="117">
+        <v>111</v>
+      </c>
+      <c r="S13" s="117" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="14.25">
+      <c r="A14" s="116" t="s">
         <v>822</v>
       </c>
-      <c r="H13" s="117">
-        <v>-8641.7000000000007</v>
-      </c>
-      <c r="I13" s="117">
-        <v>398</v>
-      </c>
-      <c r="J13" s="117" t="s">
-        <v>822</v>
-      </c>
-      <c r="K13" s="117">
-        <v>-2978.8</v>
-      </c>
-      <c r="L13" s="117">
-        <v>139.80000000000001</v>
-      </c>
-      <c r="M13" s="117" t="s">
-        <v>822</v>
-      </c>
-      <c r="N13" s="117">
-        <v>-2459.9</v>
-      </c>
-      <c r="O13" s="117">
-        <v>111</v>
-      </c>
-      <c r="P13" s="117" t="s">
-        <v>822</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="14.25">
-      <c r="A14" s="116" t="s">
-        <v>823</v>
-      </c>
       <c r="B14" s="117">
-        <v>-102.8</v>
+        <v>16.3</v>
       </c>
       <c r="C14" s="117"/>
       <c r="D14" s="117"/>
       <c r="E14" s="117">
-        <v>16.3</v>
+        <v>-102.8</v>
       </c>
       <c r="F14" s="117"/>
       <c r="G14" s="117"/>
       <c r="H14" s="117">
-        <v>-91.8</v>
+        <v>16.3</v>
       </c>
       <c r="I14" s="117"/>
       <c r="J14" s="117"/>
       <c r="K14" s="117">
-        <v>-239.6</v>
+        <v>-91.8</v>
       </c>
       <c r="L14" s="117"/>
       <c r="M14" s="117"/>
       <c r="N14" s="117">
-        <v>-63.4</v>
+        <v>-239.6</v>
       </c>
       <c r="O14" s="117"/>
       <c r="P14" s="117"/>
-    </row>
-    <row r="15" spans="1:16" ht="14.25">
+      <c r="Q14" s="117">
+        <v>-63.4</v>
+      </c>
+      <c r="R14" s="117"/>
+      <c r="S14" s="117"/>
+    </row>
+    <row r="15" spans="1:19" ht="14.25">
       <c r="A15" s="116" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B15" s="117">
-        <v>118.3</v>
+        <v>543.6</v>
       </c>
       <c r="C15" s="117"/>
       <c r="D15" s="117"/>
       <c r="E15" s="117">
-        <v>543.6</v>
+        <v>118.3</v>
       </c>
       <c r="F15" s="117"/>
       <c r="G15" s="117"/>
       <c r="H15" s="117">
-        <v>109.5</v>
+        <v>543.6</v>
       </c>
       <c r="I15" s="117"/>
       <c r="J15" s="117"/>
       <c r="K15" s="117">
-        <v>264.10000000000002</v>
+        <v>109.5</v>
       </c>
       <c r="L15" s="117"/>
       <c r="M15" s="117"/>
       <c r="N15" s="117">
-        <v>155.6</v>
+        <v>264.10000000000002</v>
       </c>
       <c r="O15" s="117"/>
       <c r="P15" s="117"/>
-    </row>
-    <row r="16" spans="1:16" ht="14.25">
+      <c r="Q15" s="117">
+        <v>155.6</v>
+      </c>
+      <c r="R15" s="117"/>
+      <c r="S15" s="117"/>
+    </row>
+    <row r="16" spans="1:19" ht="14.25">
       <c r="A16" s="116" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B16" s="117">
-        <v>-11014</v>
+        <v>-6121.5</v>
       </c>
       <c r="C16" s="117"/>
       <c r="D16" s="117"/>
       <c r="E16" s="117">
-        <v>-6121.5</v>
+        <v>-11014</v>
       </c>
       <c r="F16" s="117"/>
       <c r="G16" s="117"/>
       <c r="H16" s="117">
-        <v>-10859</v>
+        <v>-6121.5</v>
       </c>
       <c r="I16" s="117"/>
       <c r="J16" s="117"/>
       <c r="K16" s="117">
-        <v>-10386.299999999999</v>
+        <v>-10859</v>
       </c>
       <c r="L16" s="117"/>
       <c r="M16" s="117"/>
       <c r="N16" s="117">
-        <v>-10382</v>
+        <v>-10386.299999999999</v>
       </c>
       <c r="O16" s="117"/>
       <c r="P16" s="117"/>
-    </row>
-    <row r="17" spans="1:16" ht="14.25">
+      <c r="Q16" s="117">
+        <v>-10382</v>
+      </c>
+      <c r="R16" s="117"/>
+      <c r="S16" s="117"/>
+    </row>
+    <row r="17" spans="1:19" ht="14.25">
       <c r="A17" s="116" t="s">
-        <v>826</v>
-      </c>
-      <c r="B17" s="117"/>
+        <v>825</v>
+      </c>
+      <c r="B17" s="117">
+        <v>-1927.1</v>
+      </c>
       <c r="C17" s="117"/>
       <c r="D17" s="117"/>
-      <c r="E17" s="117">
-        <v>-1927.1</v>
-      </c>
+      <c r="E17" s="117"/>
       <c r="F17" s="117"/>
       <c r="G17" s="117"/>
-      <c r="H17" s="117"/>
+      <c r="H17" s="117">
+        <v>-1927.1</v>
+      </c>
       <c r="I17" s="117"/>
       <c r="J17" s="117"/>
-      <c r="K17" s="117">
-        <v>-14290.6</v>
-      </c>
+      <c r="K17" s="117"/>
       <c r="L17" s="117"/>
       <c r="M17" s="117"/>
       <c r="N17" s="117">
-        <v>-17193.099999999999</v>
+        <v>-14290.6</v>
       </c>
       <c r="O17" s="117"/>
       <c r="P17" s="117"/>
+      <c r="Q17" s="117">
+        <v>-17193.099999999999</v>
+      </c>
+      <c r="R17" s="117"/>
+      <c r="S17" s="117"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="E1:G1"/>
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="K1:M1"/>
     <mergeCell ref="N1:P1"/>
+    <mergeCell ref="Q1:S1"/>
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
-  <conditionalFormatting sqref="B3:P17">
+  <conditionalFormatting sqref="B3:S17">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>